<commit_message>
fix(upload): add seamless local file storage fallback in CloudinaryService and configure application-local
</commit_message>
<xml_diff>
--- a/NOP_BAI_DO_AN/5_Bang_Tu_Cham_Diem_Google_Sheet_Mau.xlsx
+++ b/NOP_BAI_DO_AN/5_Bang_Tu_Cham_Diem_Google_Sheet_Mau.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Spring Boot 4, Java 21, Thymeleaf, Bootstrap 5, Spring Data JPA, SQL Server 2022, Spring Security + JWT, WebSocket STOMP, Cloudinary, AI Chatbot, Docker + CI/CD</t>
+          <t>Spring Boot 4, Java 21, Thymeleaf, Bootstrap 5, Spring Data JPA, SQL Server 2022, Spring Security + JWT, WebSocket STOMP, Cloudinary, AI Chatbot</t>
         </is>
       </c>
       <c r="C4" s="2" t="n"/>
@@ -713,7 +713,7 @@
 - Đăng ký tài khoản xác thực OTP qua Email (Gmail SMTP), Quên mật khẩu / Đặt lại mật khẩu.
 - Tích hợp Cloudinary API upload hình ảnh/video lên đám mây.
 - Phân hệ Admin Hệ thống &amp; Manager Vận hành chuỗi: Dashboard toàn chuỗi, Xuất báo cáo doanh thu Excel, Quản lý người dùng &amp; khóa/mở khóa, Quản lý Chi nhánh, Danh mục, Chiết khấu hoa hồng (Commission), Mã giảm giá (Voucher), Đơn vị vận chuyển.
-- Thiết kế CSDL SQL Server 23 bảng chuẩn Unicode NVARCHAR + DevOps (Multi-stage Dockerfile, docker-compose, GitHub Actions CI/CD) + Tổng hợp code &amp; Báo cáo.</t>
+- Thiết kế CSDL SQL Server 23 bảng chuẩn Unicode NVARCHAR + Tổng hợp code &amp; Báo cáo.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">

</xml_diff>